<commit_message>
Remove outdated prediction configurations and dataset files for FXN_0701 and FXN_0703. This includes the deletion of plans.json, predict_from_raw_data_args.json, and dataset.json files, streamlining the project structure and ensuring only relevant data is retained for ongoing work.
</commit_message>
<xml_diff>
--- a/Data/FXN_2023_new（GC）/ATP.xlsx
+++ b/Data/FXN_2023_new（GC）/ATP.xlsx
@@ -1,36 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\student\Private\student11\Measure\Measure_copy\Data\FXN_2023_new\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E07A949C-0660-48A5-A5DD-BAC3E64EB6E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -40,6 +16,24 @@
     <t>Name</t>
   </si>
   <si>
+    <t>PC1</t>
+  </si>
+  <si>
+    <t>PC2</t>
+  </si>
+  <si>
+    <t>PC3</t>
+  </si>
+  <si>
+    <t>PC4</t>
+  </si>
+  <si>
+    <t>Result_Score</t>
+  </si>
+  <si>
+    <t>ATP</t>
+  </si>
+  <si>
     <t>C10_0701</t>
   </si>
   <si>
@@ -146,68 +140,33 @@
   </si>
   <si>
     <t>F9_0701</t>
-  </si>
-  <si>
-    <t>Result_Score</t>
-  </si>
-  <si>
-    <t>PC1</t>
-  </si>
-  <si>
-    <t>PC2</t>
-  </si>
-  <si>
-    <t>PC3</t>
-  </si>
-  <si>
-    <t>PC4</t>
-  </si>
-  <si>
-    <t>ATP</t>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <family val="2"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="等线"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
       <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="等线"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -228,41 +187,37 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="常规 2" xfId="1" xr:uid="{5661C1C1-DD67-48D8-96AD-60B3E2A89848}"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -288,44 +243,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -355,12 +310,12 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -399,676 +354,731 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O37"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H37"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="6" max="6" width="15.625" customWidth="1"/>
-    <col min="13" max="13" width="12.25" customWidth="1"/>
-    <col min="15" max="15" width="9.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="5" width="13.571428571428571" customWidth="1"/>
+    <col min="6" max="6" width="15.571428571428571" customWidth="1"/>
+    <col min="7" max="7" width="13.571428571428571" customWidth="1"/>
+    <col min="8" max="8" width="9.571428571428571" customWidth="1"/>
+    <col min="9" max="17" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>41</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="O1" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B2">
-        <v>5.2980282223563133</v>
+        <v>5.298028222356313</v>
       </c>
       <c r="C2">
-        <v>-3.0524812625070492</v>
+        <v>-3.052481262507049</v>
       </c>
       <c r="D2">
-        <v>-6.1399126227675183</v>
+        <v>-6.139912622767518</v>
       </c>
       <c r="E2">
         <v>0.9145291457170972</v>
       </c>
       <c r="F2">
-        <v>0.82442272913346115</v>
-      </c>
-      <c r="O2" s="3">
+        <v>0.8244227291334612</v>
+      </c>
+      <c r="H2" s="3">
         <v>54230</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B3">
-        <v>6.5061118901043367</v>
+        <v>6.506111890104337</v>
       </c>
       <c r="C3">
-        <v>-5.9593001246935424</v>
+        <v>-5.959300124693542</v>
       </c>
       <c r="D3">
-        <v>-5.5730949826581968</v>
+        <v>-5.573094982658197</v>
       </c>
       <c r="E3">
-        <v>0.28343178356539822</v>
+        <v>0.2834317835653982</v>
       </c>
       <c r="F3">
-        <v>0.69026469035809734</v>
-      </c>
-      <c r="O3" s="3">
+        <v>0.6902646903580973</v>
+      </c>
+      <c r="H3" s="3">
         <v>24330</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B4">
-        <v>15.365865549365891</v>
+        <v>15.36586554936589</v>
       </c>
       <c r="C4">
         <v>-2.673670214485647</v>
       </c>
       <c r="D4">
-        <v>-4.4641378059746808</v>
+        <v>-4.464137805974681</v>
       </c>
       <c r="E4">
-        <v>-6.8632502289114488</v>
+        <v>-6.863250228911449</v>
       </c>
       <c r="F4">
-        <v>4.9743833472158121</v>
-      </c>
-      <c r="O4" s="3">
+        <v>4.974383347215812</v>
+      </c>
+      <c r="H4" s="3">
         <v>71930</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B5">
         <v>15.22385052641784</v>
       </c>
       <c r="C5">
-        <v>-2.7692544863860591</v>
+        <v>-2.769254486386059</v>
       </c>
       <c r="D5">
-        <v>-5.4150368054041564</v>
+        <v>-5.415036805404156</v>
       </c>
       <c r="E5">
-        <v>-6.6796000357268586</v>
+        <v>-6.679600035726859</v>
       </c>
       <c r="F5">
-        <v>4.7495371146565439</v>
-      </c>
-      <c r="O5" s="3">
+        <v>4.749537114656544</v>
+      </c>
+      <c r="H5" s="3">
         <v>2961000</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B6">
-        <v>2.9810060278543871</v>
+        <v>2.981006027854387</v>
       </c>
       <c r="C6">
-        <v>-0.66110544486887446</v>
+        <v>-0.6611054448688745</v>
       </c>
       <c r="D6">
-        <v>-7.7214776356516941</v>
+        <v>-7.721477635651694</v>
       </c>
       <c r="E6">
-        <v>0.49875247846380649</v>
+        <v>0.4987524784638065</v>
       </c>
       <c r="F6">
-        <v>1.9120359889938321E-2</v>
-      </c>
-      <c r="O6" s="3">
+        <v>0.01912035988993832</v>
+      </c>
+      <c r="H6" s="3">
         <v>6731000</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B7">
-        <v>13.934673189225551</v>
+        <v>13.93467318922555</v>
       </c>
       <c r="C7">
-        <v>-1.2425666743732351</v>
+        <v>-1.242566674373235</v>
       </c>
       <c r="D7">
-        <v>-6.5390468924393774</v>
+        <v>-6.539046892439377</v>
       </c>
       <c r="E7">
-        <v>-8.4509441791259334</v>
+        <v>-8.450944179125933</v>
       </c>
       <c r="F7">
-        <v>4.1247611427306907</v>
-      </c>
-      <c r="O7" s="3">
+        <v>4.124761142730691</v>
+      </c>
+      <c r="H7" s="3">
         <v>8638000</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B8">
         <v>0.725899580521844</v>
       </c>
       <c r="C8">
-        <v>-0.87312772077231504</v>
+        <v>-0.873127720772315</v>
       </c>
       <c r="D8">
-        <v>-10.481421384104189</v>
+        <v>-10.48142138410419</v>
       </c>
       <c r="E8">
         <v>3.754783387446603</v>
       </c>
       <c r="F8">
-        <v>-1.1533090328669531</v>
-      </c>
-      <c r="O8" s="3">
+        <v>-1.153309032866953</v>
+      </c>
+      <c r="H8" s="3">
         <v>7800000</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B9">
-        <v>13.606941985466539</v>
+        <v>13.60694198546654</v>
       </c>
       <c r="C9">
-        <v>-0.66010913036630836</v>
+        <v>-0.6601091303663084</v>
       </c>
       <c r="D9">
-        <v>-5.8161096342151302</v>
+        <v>-5.81610963421513</v>
       </c>
       <c r="E9">
-        <v>-8.8874049995569511</v>
+        <v>-8.887404999556951</v>
       </c>
       <c r="F9">
         <v>4.181901924623471</v>
       </c>
-      <c r="O9" s="3">
+      <c r="H9" s="3">
         <v>7260000</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B10">
-        <v>2.3244474739587968</v>
+        <v>2.324447473958797</v>
       </c>
       <c r="C10">
-        <v>-8.015210704728977E-2</v>
+        <v>-0.08015210704728977</v>
       </c>
       <c r="D10">
-        <v>-7.9804306924331314</v>
+        <v>-7.980430692433131</v>
       </c>
       <c r="E10">
-        <v>1.1990767158270439</v>
+        <v>1.199076715827044</v>
       </c>
       <c r="F10">
-        <v>-0.10351470248234169</v>
-      </c>
-      <c r="O10" s="3">
+        <v>-0.1035147024823417</v>
+      </c>
+      <c r="H10" s="3">
         <v>6671000</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B11">
-        <v>4.5815342816880804</v>
+        <v>4.58153428168808</v>
       </c>
       <c r="C11">
-        <v>-1.5997324185104489</v>
+        <v>-1.599732418510449</v>
       </c>
       <c r="D11">
-        <v>-7.8475628583707806</v>
+        <v>-7.847562858370781</v>
       </c>
       <c r="E11">
-        <v>-4.2227131127052918E-2</v>
+        <v>-0.04222713112705292</v>
       </c>
       <c r="F11">
         <v>0.4510801230295558</v>
       </c>
-      <c r="O11" s="3">
+      <c r="H11" s="3">
         <v>77960</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B12">
-        <v>3.4651355537633211</v>
+        <v>3.465135553763321</v>
       </c>
       <c r="C12">
-        <v>-0.45374790707072421</v>
+        <v>-0.4537479070707242</v>
       </c>
       <c r="D12">
-        <v>-9.4989870866684107</v>
+        <v>-9.49898708666841</v>
       </c>
       <c r="E12">
-        <v>-0.20517812324404039</v>
+        <v>-0.2051781232440404</v>
       </c>
       <c r="F12">
-        <v>-8.0651156764439458E-2</v>
-      </c>
-      <c r="O12" s="3">
+        <v>-0.08065115676443946</v>
+      </c>
+      <c r="H12" s="3">
         <v>185300</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B13">
-        <v>2.7793018231422568</v>
+        <v>2.779301823142257</v>
       </c>
       <c r="C13">
         <v>-2.618510827621134</v>
       </c>
       <c r="D13">
-        <v>-8.7778868219783313</v>
+        <v>-8.777886821978331</v>
       </c>
       <c r="E13">
-        <v>6.3954299796845051</v>
+        <v>6.395429979684505</v>
       </c>
       <c r="F13">
-        <v>-2.4768930496542271E-2</v>
-      </c>
-      <c r="O13" s="3">
+        <v>-0.02476893049654227</v>
+      </c>
+      <c r="H13" s="3">
         <v>46930</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B14">
-        <v>17.023383112082641</v>
+        <v>17.02338311208264</v>
       </c>
       <c r="C14">
-        <v>-4.7382555420022854</v>
+        <v>-4.738255542002285</v>
       </c>
       <c r="D14">
-        <v>-1.9731815324074591</v>
+        <v>-1.973181532407459</v>
       </c>
       <c r="E14">
-        <v>-5.4631015031722843</v>
+        <v>-5.463101503172284</v>
       </c>
       <c r="F14">
-        <v>5.8197014899186179</v>
-      </c>
-      <c r="O14" s="3">
+        <v>5.819701489918618</v>
+      </c>
+      <c r="H14" s="3">
         <v>45350</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B15">
-        <v>14.433816389404861</v>
+        <v>14.43381638940486</v>
       </c>
       <c r="C15">
-        <v>-2.0337572655762099</v>
+        <v>-2.03375726557621</v>
       </c>
       <c r="D15">
-        <v>-4.9094877207326846</v>
+        <v>-4.909487720732685</v>
       </c>
       <c r="E15">
-        <v>-8.2882354670930596</v>
+        <v>-8.28823546709306</v>
       </c>
       <c r="F15">
         <v>4.451427892190515</v>
       </c>
-      <c r="O15" s="3">
+      <c r="H15" s="3">
         <v>133600</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B16">
-        <v>2.4856599398042101</v>
+        <v>2.48565993980421</v>
       </c>
       <c r="C16">
-        <v>0.86878478315029162</v>
+        <v>0.8687847831502916</v>
       </c>
       <c r="D16">
-        <v>-6.5843691839628598</v>
+        <v>-6.58436918396286</v>
       </c>
       <c r="E16">
-        <v>-9.0339938846613038E-2</v>
+        <v>-0.09033993884661304</v>
       </c>
       <c r="F16">
-        <v>0.28161538205089548</v>
-      </c>
-      <c r="O16" s="3">
+        <v>0.2816153820508955</v>
+      </c>
+      <c r="H16" s="3">
         <v>28820</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B17">
         <v>-2.29706486610376</v>
       </c>
       <c r="C17">
-        <v>-4.2107941704188088</v>
+        <v>-4.210794170418809</v>
       </c>
       <c r="D17">
         <v>-10.18726679582722</v>
       </c>
       <c r="E17">
-        <v>9.9177291005973682</v>
+        <v>9.917729100597368</v>
       </c>
       <c r="F17">
-        <v>-2.6041529360034348</v>
-      </c>
-      <c r="O17" s="3">
+        <v>-2.604152936003435</v>
+      </c>
+      <c r="H17" s="3">
         <v>66260</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B18">
-        <v>4.1363813168513506</v>
+        <v>4.136381316851351</v>
       </c>
       <c r="C18">
-        <v>-0.88453504762806112</v>
+        <v>-0.8845350476280611</v>
       </c>
       <c r="D18">
         <v>-7.6201438516944</v>
       </c>
       <c r="E18">
-        <v>0.27465744839917178</v>
+        <v>0.2746574483991718</v>
       </c>
       <c r="F18">
-        <v>0.49473523472114639</v>
-      </c>
-      <c r="O18" s="3">
+        <v>0.4947352347211464</v>
+      </c>
+      <c r="H18" s="3">
         <v>27630</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B19">
-        <v>2.5599059533568078</v>
+        <v>2.559905953356808</v>
       </c>
       <c r="C19">
-        <v>-1.2467879175093011</v>
+        <v>-1.246787917509301</v>
       </c>
       <c r="D19">
-        <v>-7.8589889977083613</v>
+        <v>-7.858988997708361</v>
       </c>
       <c r="E19">
-        <v>0.89776407535572011</v>
+        <v>0.8977640753557201</v>
       </c>
       <c r="F19">
         <v>-0.297382635201767</v>
       </c>
-      <c r="O19" s="3">
+      <c r="H19" s="3">
         <v>25920</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B20">
         <v>14.8334153275687</v>
       </c>
       <c r="C20">
-        <v>0.29892901942482869</v>
+        <v>0.2989290194248287</v>
       </c>
       <c r="D20">
-        <v>-3.2469726465471398</v>
+        <v>-3.24697264654714</v>
       </c>
       <c r="E20">
-        <v>-6.4245842681216976</v>
+        <v>-6.424584268121698</v>
       </c>
       <c r="F20">
-        <v>5.7122013950861197</v>
-      </c>
-      <c r="O20" s="3">
+        <v>5.71220139508612</v>
+      </c>
+      <c r="H20" s="3">
         <v>32980</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B21">
-        <v>13.720577827492409</v>
+        <v>13.72057782749241</v>
       </c>
       <c r="C21">
-        <v>-0.56663908495719639</v>
+        <v>-0.5666390849571964</v>
       </c>
       <c r="D21">
-        <v>-4.4719463676740281</v>
+        <v>-4.471946367674028</v>
       </c>
       <c r="E21">
-        <v>-7.1215528068595004</v>
+        <v>-7.1215528068595</v>
       </c>
       <c r="F21">
-        <v>4.6918325564444192</v>
-      </c>
-      <c r="O21" s="3">
+        <v>4.691832556444419</v>
+      </c>
+      <c r="H21" s="3">
         <v>51460</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B22">
-        <v>13.379291578278069</v>
+        <v>13.37929157827807</v>
       </c>
       <c r="C22">
-        <v>0.32429595174758907</v>
+        <v>0.3242959517475891</v>
       </c>
       <c r="D22">
-        <v>-4.1302195527139522</v>
+        <v>-4.130219552713952</v>
       </c>
       <c r="E22">
-        <v>-8.0266939539734796</v>
+        <v>-8.02669395397348</v>
       </c>
       <c r="F22">
         <v>4.699639696511043</v>
       </c>
-      <c r="O22" s="3">
+      <c r="H22" s="3">
         <v>69330</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B23">
-        <v>15.323822064032431</v>
+        <v>15.32382206403243</v>
       </c>
       <c r="C23">
-        <v>-5.5445212463227334</v>
+        <v>-5.544521246322733</v>
       </c>
       <c r="D23">
         <v>-3.829014290819245</v>
@@ -1077,245 +1087,245 @@
         <v>-7.226093456768381</v>
       </c>
       <c r="F23">
-        <v>4.3072506690665424</v>
-      </c>
-      <c r="O23" s="3">
+        <v>4.307250669066542</v>
+      </c>
+      <c r="H23" s="3">
         <v>63070</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B24">
-        <v>5.1275638269862611</v>
+        <v>5.127563826986261</v>
       </c>
       <c r="C24">
-        <v>-6.7716831297239519</v>
+        <v>-6.771683129723952</v>
       </c>
       <c r="D24">
-        <v>-6.3039727750686074</v>
+        <v>-6.303972775068607</v>
       </c>
       <c r="E24">
         <v>1.015331354742292</v>
       </c>
       <c r="F24">
-        <v>-0.18836659909045331</v>
-      </c>
-      <c r="O24" s="3">
+        <v>-0.1883665990904533</v>
+      </c>
+      <c r="H24" s="3">
         <v>15450</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B25">
-        <v>14.425711780467751</v>
+        <v>14.42571178046775</v>
       </c>
       <c r="C25">
-        <v>0.27676467732017662</v>
+        <v>0.2767646773201766</v>
       </c>
       <c r="D25">
-        <v>-5.5858990410214684</v>
+        <v>-5.585899041021468</v>
       </c>
       <c r="E25">
-        <v>-7.4672526324052582</v>
+        <v>-7.467252632405258</v>
       </c>
       <c r="F25">
-        <v>5.0049650073814256</v>
-      </c>
-      <c r="O25" s="3">
+        <v>5.004965007381426</v>
+      </c>
+      <c r="H25" s="3">
         <v>68250</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B26">
-        <v>14.410043441683021</v>
+        <v>14.41004344168302</v>
       </c>
       <c r="C26">
-        <v>-2.2082641265233418</v>
+        <v>-2.208264126523342</v>
       </c>
       <c r="D26">
-        <v>-4.0306229309421262</v>
+        <v>-4.030622930942126</v>
       </c>
       <c r="E26">
-        <v>-7.7123163496613643</v>
+        <v>-7.712316349661364</v>
       </c>
       <c r="F26">
-        <v>4.6112924822510486</v>
-      </c>
-      <c r="O26" s="3">
+        <v>4.611292482251049</v>
+      </c>
+      <c r="H26" s="3">
         <v>56050000</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B27">
-        <v>6.5290462690763178</v>
+        <v>6.529046269076318</v>
       </c>
       <c r="C27">
-        <v>-6.0417094510662608</v>
+        <v>-6.041709451066261</v>
       </c>
       <c r="D27">
-        <v>-5.0694861859330587</v>
+        <v>-5.069486185933059</v>
       </c>
       <c r="E27">
         <v>1.727443360013482</v>
       </c>
       <c r="F27">
-        <v>0.93706598421197906</v>
-      </c>
-      <c r="O27" s="3">
+        <v>0.9370659842119791</v>
+      </c>
+      <c r="H27" s="3">
         <v>55300000</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B28">
-        <v>4.6891390516166593</v>
+        <v>4.689139051616659</v>
       </c>
       <c r="C28">
-        <v>-2.8816108658225348</v>
+        <v>-2.881610865822535</v>
       </c>
       <c r="D28">
-        <v>-6.2094674391041966</v>
+        <v>-6.209467439104197</v>
       </c>
       <c r="E28">
-        <v>2.0420477662116729</v>
+        <v>2.042047766211673</v>
       </c>
       <c r="F28">
-        <v>0.70540310857260569</v>
-      </c>
-      <c r="O28" s="3">
+        <v>0.7054031085726057</v>
+      </c>
+      <c r="H28" s="3">
         <v>46400000</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B29">
-        <v>17.050792324698151</v>
+        <v>17.05079232469815</v>
       </c>
       <c r="C29">
         <v>-4.858292877798922</v>
       </c>
       <c r="D29">
-        <v>-2.9916121779548219</v>
+        <v>-2.991612177954822</v>
       </c>
       <c r="E29">
-        <v>-5.5194723141017343</v>
+        <v>-5.519472314101734</v>
       </c>
       <c r="F29">
-        <v>5.6281940395241028</v>
-      </c>
-      <c r="O29" s="3">
+        <v>5.628194039524103</v>
+      </c>
+      <c r="H29" s="3">
         <v>12407000</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B30">
-        <v>13.878540661382431</v>
+        <v>13.87854066138243</v>
       </c>
       <c r="C30">
-        <v>-1.2753771211151561</v>
+        <v>-1.275377121115156</v>
       </c>
       <c r="D30">
-        <v>-3.2371287963319211</v>
+        <v>-3.237128796331921</v>
       </c>
       <c r="E30">
-        <v>-8.9566993614385524</v>
+        <v>-8.956699361438552</v>
       </c>
       <c r="F30">
         <v>4.574165357825267</v>
       </c>
-      <c r="O30" s="3">
+      <c r="H30" s="3">
         <v>14970000</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B31">
-        <v>4.1111597001072262</v>
+        <v>4.111159700107226</v>
       </c>
       <c r="C31">
-        <v>-4.4062772314026084</v>
+        <v>-4.406277231402608</v>
       </c>
       <c r="D31">
-        <v>-7.2905191211342917</v>
+        <v>-7.290519121134292</v>
       </c>
       <c r="E31">
-        <v>-4.0488690877845387E-2</v>
+        <v>-0.04048869087784539</v>
       </c>
       <c r="F31">
-        <v>-0.36983505636483072</v>
-      </c>
-      <c r="O31" s="3">
+        <v>-0.3698350563648307</v>
+      </c>
+      <c r="H31" s="3">
         <v>14070000</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B32">
-        <v>5.6834870969950781</v>
+        <v>5.683487096995078</v>
       </c>
       <c r="C32">
-        <v>-2.5937684071361269</v>
+        <v>-2.593768407136127</v>
       </c>
       <c r="D32">
-        <v>-6.3909206636086999</v>
+        <v>-6.3909206636087</v>
       </c>
       <c r="E32">
         <v>0.2780048878823867</v>
       </c>
       <c r="F32">
-        <v>1.0003151716882179</v>
-      </c>
-      <c r="O32" s="3">
+        <v>1.000315171688218</v>
+      </c>
+      <c r="H32" s="3">
         <v>10820000</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B33">
-        <v>3.5219868013022331</v>
+        <v>3.521986801302233</v>
       </c>
       <c r="C33">
-        <v>-1.9512034730905541</v>
+        <v>-1.951203473090554</v>
       </c>
       <c r="D33">
-        <v>-6.5276052802094426</v>
+        <v>-6.527605280209443</v>
       </c>
       <c r="E33">
-        <v>2.3556850160905638</v>
+        <v>2.355685016090564</v>
       </c>
       <c r="F33">
-        <v>0.37377769465610838</v>
-      </c>
-      <c r="O33" s="3">
+        <v>0.3737776946561084</v>
+      </c>
+      <c r="H33" s="3">
         <v>6017000</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B34">
         <v>11.99664057935721</v>
@@ -1324,90 +1334,89 @@
         <v>6.873275189449024</v>
       </c>
       <c r="D34">
-        <v>-5.4668772241518946</v>
+        <v>-5.466877224151895</v>
       </c>
       <c r="E34">
-        <v>-8.6981906141820247</v>
+        <v>-8.698190614182025</v>
       </c>
       <c r="F34">
-        <v>5.3677409741038193</v>
-      </c>
-      <c r="O34" s="3">
+        <v>5.367740974103819</v>
+      </c>
+      <c r="H34" s="3">
         <v>12140000</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B35">
         <v>15.42935687496394</v>
       </c>
       <c r="C35">
-        <v>-5.3135153960241599</v>
+        <v>-5.31351539602416</v>
       </c>
       <c r="D35">
-        <v>-2.1006570031805141</v>
+        <v>-2.100657003180514</v>
       </c>
       <c r="E35">
-        <v>-6.9852680072819284</v>
+        <v>-6.985268007281928</v>
       </c>
       <c r="F35">
-        <v>4.7276089794016407</v>
-      </c>
-      <c r="O35" s="3">
+        <v>4.727608979401641</v>
+      </c>
+      <c r="H35" s="3">
         <v>54140000</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B36">
         <v>14.1830821865339</v>
       </c>
       <c r="C36">
-        <v>-1.9831524050174549</v>
+        <v>-1.983152405017455</v>
       </c>
       <c r="D36">
-        <v>-5.6581128616487053</v>
+        <v>-5.658112861648705</v>
       </c>
       <c r="E36">
-        <v>-8.4336790986716785</v>
+        <v>-8.433679098671679</v>
       </c>
       <c r="F36">
-        <v>4.2056100896170587</v>
-      </c>
-      <c r="O36" s="3">
+        <v>4.205610089617059</v>
+      </c>
+      <c r="H36" s="3">
         <v>50680000</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B37">
         <v>16.25656065506967</v>
       </c>
       <c r="C37">
-        <v>-5.3516059796849378</v>
+        <v>-5.351605979684938</v>
       </c>
       <c r="D37">
-        <v>-3.1829956331802349</v>
+        <v>-3.182995633180235</v>
       </c>
       <c r="E37">
-        <v>-7.0779139765035151</v>
+        <v>-7.077913976503515</v>
       </c>
       <c r="F37">
         <v>4.915906381984362</v>
       </c>
-      <c r="O37" s="3">
+      <c r="H37" s="3">
         <v>65380000</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>